<commit_message>
add excel di linux e add progetto di libereria en clena architecture
</commit_message>
<xml_diff>
--- a/Linux/Commands.xlsx
+++ b/Linux/Commands.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\brian\Desktop\Esercizi-personali\Linux\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A69123BA-B020-4CCE-99E4-2EA08B3DF83B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA8A1B77-F62E-46B2-A51B-12ED7C67DAAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="24240" yWindow="4095" windowWidth="23430" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="615" yWindow="3765" windowWidth="23430" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t>find</t>
   </si>
@@ -64,6 +64,48 @@
   </si>
   <si>
     <t>u, g, o =&gt; +-</t>
+  </si>
+  <si>
+    <t>hostname</t>
+  </si>
+  <si>
+    <t>df -h</t>
+  </si>
+  <si>
+    <t>umask</t>
+  </si>
+  <si>
+    <t>getent group o passwd o altro</t>
+  </si>
+  <si>
+    <t>id utente</t>
+  </si>
+  <si>
+    <t>groups</t>
+  </si>
+  <si>
+    <t>sudo chgrp gruppo cartella</t>
+  </si>
+  <si>
+    <t>sudo chmod 2770 cartella</t>
+  </si>
+  <si>
+    <t>sudo groupadd grupo</t>
+  </si>
+  <si>
+    <t>sudo useradd -m -s/bin/bash -g hosp-med med.nome</t>
+  </si>
+  <si>
+    <t>which program</t>
+  </si>
+  <si>
+    <t>sudo setfacl -m g:hosp-nur:rx /srv/hospital/emr</t>
+  </si>
+  <si>
+    <t>sudo getfacl /srv</t>
+  </si>
+  <si>
+    <t>il primo puo essere 2,4 o 1</t>
   </si>
 </sst>
 </file>
@@ -381,8 +423,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="35.28515625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -447,6 +492,74 @@
         <v>12</v>
       </c>
     </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>20</v>
+      </c>
+      <c r="B22" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>25</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>